<commit_message>
Update tabelle e file excel
</commit_message>
<xml_diff>
--- a/DatiExcel/tipi_visita_vetportal.xlsx
+++ b/DatiExcel/tipi_visita_vetportal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andrea.chiampo\Desktop\LearningByProject\DatiExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C866F91E-8EA2-49BA-8193-B5C676D9DECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A3BEC06-F9D4-4943-BFD3-6484E607872F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="34350" windowHeight="16770" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="37110" windowHeight="19710" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tipi di Visita" sheetId="1" r:id="rId1"/>
@@ -322,10 +322,10 @@
     <t>Da implementare nel backend</t>
   </si>
   <si>
-    <t>Aggiungere sempre una vaccino antirabica scaduto di default</t>
-  </si>
-  <si>
     <t>Da chiedere a Scassillo</t>
+  </si>
+  <si>
+    <t>Alert Scheda Animale</t>
   </si>
 </sst>
 </file>
@@ -397,7 +397,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="26">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -515,12 +515,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor rgb="FFE8F5E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -534,12 +528,6 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor rgb="FFF5F5F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -600,7 +588,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -699,24 +687,6 @@
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -730,18 +700,30 @@
     <xf numFmtId="0" fontId="4" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1019,24 +1001,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="43" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
     </row>
     <row r="2" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
     </row>
     <row r="3" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -1075,7 +1057,7 @@
       <c r="E5" s="4">
         <v>55</v>
       </c>
-      <c r="F5" s="43" t="s">
+      <c r="F5" s="37" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1131,7 +1113,7 @@
       <c r="E8" s="7">
         <v>65</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="34" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1187,7 +1169,7 @@
       <c r="E11" s="10">
         <v>40</v>
       </c>
-      <c r="F11" s="47" t="s">
+      <c r="F11" s="40" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1261,7 +1243,7 @@
       <c r="E15" s="10">
         <v>30</v>
       </c>
-      <c r="F15" s="45" t="s">
+      <c r="F15" s="40" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1281,7 +1263,7 @@
       <c r="E16" s="7">
         <v>25</v>
       </c>
-      <c r="F16" s="49" t="s">
+      <c r="F16" s="34" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1356,9 +1338,9 @@
         <v>25</v>
       </c>
       <c r="F20" s="6"/>
-      <c r="H20" s="50"/>
-      <c r="I20" s="50" t="s">
-        <v>93</v>
+      <c r="H20" s="42"/>
+      <c r="I20" s="42" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1378,8 +1360,8 @@
         <v>60</v>
       </c>
       <c r="F21" s="12"/>
-      <c r="H21" s="46"/>
-      <c r="I21" s="46" t="s">
+      <c r="H21" s="39"/>
+      <c r="I21" s="39" t="s">
         <v>91</v>
       </c>
     </row>
@@ -1399,11 +1381,11 @@
       <c r="E22" s="7">
         <v>45</v>
       </c>
-      <c r="F22" s="49" t="s">
+      <c r="F22" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="H22" s="42"/>
-      <c r="I22" s="42" t="s">
+      <c r="H22" s="36"/>
+      <c r="I22" s="36" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1424,9 +1406,9 @@
         <v>35</v>
       </c>
       <c r="F23" s="12"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="48" t="s">
-        <v>92</v>
+      <c r="H23" s="41"/>
+      <c r="I23" s="41" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1553,7 +1535,7 @@
       <c r="E30" s="7">
         <v>130</v>
       </c>
-      <c r="F30" s="40" t="s">
+      <c r="F30" s="34" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1573,7 +1555,7 @@
       <c r="E31" s="22">
         <v>180</v>
       </c>
-      <c r="F31" s="41" t="s">
+      <c r="F31" s="35" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1593,7 +1575,7 @@
       <c r="E32" s="7">
         <v>120</v>
       </c>
-      <c r="F32" s="40"/>
+      <c r="F32" s="34"/>
     </row>
     <row r="33" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="20">
@@ -1611,7 +1593,7 @@
       <c r="E33" s="22">
         <v>250</v>
       </c>
-      <c r="F33" s="41" t="s">
+      <c r="F33" s="35" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1631,7 +1613,7 @@
       <c r="E34" s="7">
         <v>320</v>
       </c>
-      <c r="F34" s="40" t="s">
+      <c r="F34" s="34" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1651,7 +1633,7 @@
       <c r="E35" s="22">
         <v>400</v>
       </c>
-      <c r="F35" s="41" t="s">
+      <c r="F35" s="35" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1833,16 +1815,16 @@
       <c r="E45" s="28">
         <v>110</v>
       </c>
-      <c r="F45" s="44" t="s">
+      <c r="F45" s="38" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="36" t="s">
+      <c r="A46" s="45" t="s">
         <v>64</v>
       </c>
-      <c r="B46" s="36"/>
-      <c r="C46" s="36"/>
+      <c r="B46" s="45"/>
+      <c r="C46" s="45"/>
       <c r="D46" s="29">
         <f>AVERAGE(D5:D45)</f>
         <v>31.707317073170731</v>
@@ -1875,11 +1857,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="32" t="s">
@@ -1959,48 +1941,48 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="47" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
     </row>
     <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="39" t="s">
+      <c r="A11" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
     </row>
     <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="39"/>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
+      <c r="A12" s="48"/>
+      <c r="B12" s="48"/>
+      <c r="C12" s="48"/>
     </row>
     <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="39"/>
-      <c r="B13" s="39"/>
-      <c r="C13" s="39"/>
+      <c r="A13" s="48"/>
+      <c r="B13" s="48"/>
+      <c r="C13" s="48"/>
     </row>
     <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="39"/>
-      <c r="B14" s="39"/>
-      <c r="C14" s="39"/>
+      <c r="A14" s="48"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
     </row>
     <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="39"/>
-      <c r="B15" s="39"/>
-      <c r="C15" s="39"/>
+      <c r="A15" s="48"/>
+      <c r="B15" s="48"/>
+      <c r="C15" s="48"/>
     </row>
     <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="39"/>
-      <c r="B16" s="39"/>
-      <c r="C16" s="39"/>
+      <c r="A16" s="48"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="48"/>
     </row>
     <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="39"/>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39"/>
+      <c r="A17" s="48"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>